<commit_message>
Added the components of chassis ground to the BOM file
</commit_message>
<xml_diff>
--- a/Hardware/BLDC_MC_V1.0/Output_Job_files/BOM_File/BLDC_MC_V1.0_Excel.xlsx
+++ b/Hardware/BLDC_MC_V1.0/Output_Job_files/BOM_File/BLDC_MC_V1.0_Excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP - Victus\Desktop\Rnd\BLDC_Motor_Driver\Hardware\BLDC_MC_V1.0\Output_Job_files\BOM_File\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A19CE1-E443-4AEF-B0B7-F50624667704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB3FD03-43E8-4305-802A-E80137A74134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8D33A46B-759D-415B-9EA8-C2ABC5F69A52}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="269">
   <si>
     <t>MP</t>
   </si>
@@ -806,6 +806,27 @@
   </si>
   <si>
     <t>C273526</t>
+  </si>
+  <si>
+    <t>FRC1206J105 TS</t>
+  </si>
+  <si>
+    <t>R9</t>
+  </si>
+  <si>
+    <t>1M</t>
+  </si>
+  <si>
+    <t>C2907441</t>
+  </si>
+  <si>
+    <t>TCC1206X7R103K101DT</t>
+  </si>
+  <si>
+    <t>C14</t>
+  </si>
+  <si>
+    <t>C377055</t>
   </si>
 </sst>
 </file>
@@ -1129,7 +1150,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -1320,41 +1341,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1400,7 +1386,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1420,15 +1406,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2003,7 +1981,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.6640625" customWidth="1"/>
@@ -3382,29 +3360,81 @@
       </c>
     </row>
     <row r="54" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A54" s="7" t="s">
+      <c r="A54" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="B54" s="8">
+      <c r="B54" s="5">
         <v>1</v>
       </c>
-      <c r="C54" s="8" t="s">
+      <c r="C54" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="D54" s="8" t="s">
+      <c r="D54" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="E54" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F54" s="8" t="s">
+      <c r="E54" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F54" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="G54" s="8" t="s">
+      <c r="G54" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="H54" s="9" t="s">
+      <c r="H54" s="5" t="s">
         <v>253</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A55" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="B55" s="7">
+        <v>1</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="G55" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A56" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="B56" s="7">
+        <v>1</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H56" s="7" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>